<commit_message>
Deployed 030a333db to metadata-mismatch with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/metadata-mismatch/issues_list.xlsx
+++ b/metadata-mismatch/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C259"/>
+  <dimension ref="A1:C243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>e8414189-54c9-4311-874e-b97f9b7916ae</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://huggingface.co/datasets/HakaiInstitute/mussel-seg-1024-1024 returned status_code=429</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/kmam-ct93' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2759,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2864,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3089,12 +3089,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -3164,12 +3164,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3224,12 +3224,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3254,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3329,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3374,12 +3374,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3404,12 +3404,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3449,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3464,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3509,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3539,12 +3539,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3599,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3644,12 +3644,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3674,12 +3674,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3779,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/gsbw-bz85 status_code=502</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3824,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -3869,12 +3869,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3884,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3899,12 +3899,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3974,12 +3974,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3989,12 +3989,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4049,250 +4049,10 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>242</v>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>243</v>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>244</v>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>245</v>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>246</v>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>247</v>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>248</v>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>249</v>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="n">
-        <v>250</v>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="n">
-        <v>251</v>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="n">
-        <v>252</v>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="n">
-        <v>253</v>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="n">
-        <v>254</v>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="n">
-        <v>255</v>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="n">
-        <v>256</v>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="n">
-        <v>257</v>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C259" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>